<commit_message>
data: cierre dia 2026-07-01_1839 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/incentivo_club_faro .xlsx
+++ b/01_INPUTS/incentivo_club_faro .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F754697D-EAE1-4B33-99B0-BD690430437A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{513BEE2A-C959-4F88-97CA-CA058C18BA5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{AF0BFBE6-0CF4-4DE9-A435-B099ACB102B8}"/>
   </bookViews>
@@ -51,86 +51,10 @@
     <t>kiosco + almacén</t>
   </si>
   <si>
-    <t>alaris + finca las moras</t>
-  </si>
-  <si>
     <t>Autoservicios</t>
   </si>
   <si>
-    <t>Antares</t>
-  </si>
-  <si>
-    <t>familia smirnoff</t>
-  </si>
-  <si>
-    <t>en el periodo de mayo y junio el cliente debe comprar al menos una vez la cantidad mínima de botellas para cobertura (3 en kiosco+almacén y 6 en autoservicio)</t>
-  </si>
-  <si>
     <t>Regla</t>
-  </si>
-  <si>
-    <r>
-      <t>Familia Smirnoff:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF222222"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> Cada PDV contabiliza 1 CCC por la compra de productos Smirnoff (Vodka Nº21, Flavors, Bitter Citric), sin importar si adquiere uno, dos o los tres SKUs.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Antares:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF222222"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> Cada SKU suma 1 CCC, pero </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF222222"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>XPA y Lager botella suman doble</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF222222"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Alaris + FLM:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF222222"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> En kioskos y tradicionales, cada operación suma 1 CCC por cualquier SKU participante, sin acumular más de uno por compra.</t>
-    </r>
-  </si>
-  <si>
-    <t>incentivo Club FARO</t>
   </si>
   <si>
     <r>
@@ -148,7 +72,64 @@
     </r>
   </si>
   <si>
-    <t>PREMIOS: 1) FAMILIA SMIRNOFF (1000 MILLAS), ANTARES (1000 MILLAS) Y ALARIS +FLM (2000 MILLAS)</t>
+    <t>incentivo Club FARO (julio -Agosto)</t>
+  </si>
+  <si>
+    <t>smirnoff ice</t>
+  </si>
+  <si>
+    <t>familia gordons</t>
+  </si>
+  <si>
+    <t>Vinos Red Blends</t>
+  </si>
+  <si>
+    <t>en el periodo de julio - agosto el cliente debe comprar al menos una vez la cantidad mínima de botellas para cobertura (3 en kiosco+almacén y 6 en autoservicio)</t>
+  </si>
+  <si>
+    <r>
+      <t>Vinos Red Blends:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF222222"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> Cada SKU suma 1 CCC (80089, 74684, 44395, 71716,74735,42376 y 74737) en autoservicio con mínimo 6 botellas.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Familia gordons botella:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF222222"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> Cada PDV contabiliza 1 CCC por la compra en autoservicio (6 botellas), de productos Gordons x 700 (30139, 30075 y 30134), por cada variedad suma una cobertura, un cliente puede tener 3 máximo de cobertura</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Smirnoff ice:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF222222"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> En kioskos y tradicionales, cada variedad suma 1 CCC por cualquier SKU participante (35104, 35105,35103).</t>
+    </r>
+  </si>
+  <si>
+    <t>PREMIOS: 1) FAMILIA gordons (1000 MILLAS), Red Blends (1000 MILLAS) Y smirnoff ice (2000 MILLAS)</t>
   </si>
 </sst>
 </file>
@@ -578,14 +559,14 @@
   <cols>
     <col min="1" max="1" width="15" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="1"/>
+    <col min="3" max="3" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -593,7 +574,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D2" s="9"/>
     </row>
@@ -602,13 +583,13 @@
         <v>0</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -747,32 +728,32 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-07-02_1729 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/incentivo_club_faro .xlsx
+++ b/01_INPUTS/incentivo_club_faro .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{513BEE2A-C959-4F88-97CA-CA058C18BA5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5385A44A-537D-4E62-A554-EDE4BB8755C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{AF0BFBE6-0CF4-4DE9-A435-B099ACB102B8}"/>
   </bookViews>
@@ -597,7 +597,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="3">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="C4" s="3">
         <v>0</v>
@@ -611,13 +611,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="2">
-        <v>85</v>
+        <v>38</v>
       </c>
       <c r="C5" s="2">
+        <v>14</v>
+      </c>
+      <c r="D5" s="2">
         <v>8</v>
-      </c>
-      <c r="D5" s="2">
-        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -625,13 +625,13 @@
         <v>6</v>
       </c>
       <c r="B6" s="3">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="C6" s="3">
+        <v>14</v>
+      </c>
+      <c r="D6" s="3">
         <v>8</v>
-      </c>
-      <c r="D6" s="3">
-        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -639,13 +639,13 @@
         <v>7</v>
       </c>
       <c r="B7" s="2">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="C7" s="2">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D7" s="2">
-        <v>21</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -653,13 +653,13 @@
         <v>8</v>
       </c>
       <c r="B8" s="3">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="C8" s="3">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D8" s="3">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -667,13 +667,13 @@
         <v>9</v>
       </c>
       <c r="B9" s="2">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="C9" s="2">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D9" s="2">
-        <v>21</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -681,13 +681,13 @@
         <v>10</v>
       </c>
       <c r="B10" s="3">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="C10" s="3">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D10" s="3">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -703,13 +703,13 @@
         <v>2</v>
       </c>
       <c r="B12" s="3">
-        <v>422</v>
+        <v>212</v>
       </c>
       <c r="C12" s="3">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="D12" s="3">
-        <v>90</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -717,13 +717,13 @@
         <v>3</v>
       </c>
       <c r="B13" s="2">
-        <v>172</v>
+        <v>76</v>
       </c>
       <c r="C13" s="2">
+        <v>28</v>
+      </c>
+      <c r="D13" s="2">
         <v>16</v>
-      </c>
-      <c r="D13" s="2">
-        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-09-02_2247 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/incentivo_club_faro .xlsx
+++ b/01_INPUTS/incentivo_club_faro .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33A1D245-6CD7-4507-9F27-5B114724AE0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C9AE73-4841-4339-B7B5-C9327D7DBF0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{AF0BFBE6-0CF4-4DE9-A435-B099ACB102B8}"/>
   </bookViews>
@@ -72,23 +72,23 @@
     </r>
   </si>
   <si>
-    <t>incentivo Club FARO (julio -Agosto)</t>
-  </si>
-  <si>
-    <t>smirnoff ice</t>
-  </si>
-  <si>
-    <t>familia gordons</t>
-  </si>
-  <si>
-    <t>Vinos Red Blends</t>
-  </si>
-  <si>
-    <t>en el periodo de julio - agosto el cliente debe comprar al menos una vez la cantidad mínima de botellas para cobertura (3 en kiosco+almacén y 6 en autoservicio)</t>
+    <t>incentivo Club FARO (septiembre-octubre)</t>
+  </si>
+  <si>
+    <t>Familia Smirnoff</t>
+  </si>
+  <si>
+    <t>Blancos Dulces</t>
+  </si>
+  <si>
+    <t>familia frizze</t>
+  </si>
+  <si>
+    <t>en el periodo de septiembre - octubre el cliente debe comprar al menos una vez la cantidad mínima de botellas para cobertura (3 en kiosco+almacén y 6 en autoservicio)</t>
   </si>
   <si>
     <r>
-      <t>Vinos Red Blends:</t>
+      <t>Familia frizze:</t>
     </r>
     <r>
       <rPr>
@@ -97,12 +97,12 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t> Cada SKU suma 1 CCC (80089, 74684, 44395, 71716,74735,42376 y 74737) en autoservicio con mínimo 6 botellas.</t>
+      <t> Cada PDV contabiliza 1 CCC por la compra en autoservicio de productos frizze  (14620, 14621, 14583, 14619 y 14594), por cada pdv suma solo 1 cobertura por más que compre todas las variedades.</t>
     </r>
   </si>
   <si>
     <r>
-      <t>Familia gordons botella:</t>
+      <t>Vinos Blancos dulces:</t>
     </r>
     <r>
       <rPr>
@@ -111,12 +111,12 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t> Cada PDV contabiliza 1 CCC por la compra en autoservicio (6 botellas), de productos Gordons x 700 (30139, 30075 y 30134), por cada variedad suma una cobertura, un cliente puede tener 3 máximo de cobertura</t>
+      <t> Cada SKU suma 1 CCC (74188, 74840, 74509, 74882, 74816, 42113, 74827, 74397 y 74886) en autoservicio con mínimo 6 botellas.</t>
     </r>
   </si>
   <si>
     <r>
-      <t>Smirnoff ice:</t>
+      <t>Familia Smirnoff:</t>
     </r>
     <r>
       <rPr>
@@ -125,11 +125,11 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t> En kioskos y tradicionales, cada variedad suma 1 CCC por cualquier SKU participante (35104, 35105,35103).</t>
+      <t> En kioskos y tradicionales, suma 1 CCC por cualquier SKU participante (no entran BC y 21), no puede acumular un cliente más de una cobertura por más que haya comprado toda la variedad. Es solo en botella.</t>
     </r>
   </si>
   <si>
-    <t>PREMIOS: 1) FAMILIA gordons (1000 MILLAS), Red Blends (1000 MILLAS) Y smirnoff ice (2000 MILLAS)</t>
+    <t>PREMIOS: 1) FAMILIA Frizze (1000 MILLAS), Blancos Dulces (1000 MILLAS) Y familia smirnoff (2000 MILLAS)</t>
   </si>
 </sst>
 </file>
@@ -244,7 +244,28 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -255,6 +276,143 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>533783</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>105113</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D20C80B9-50DE-DEB5-37A9-1C1621B12FCC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9858375" y="161925"/>
+          <a:ext cx="2743583" cy="2419688"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>171451</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>38467</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>137015</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8E6098A3-F89D-7840-4223-F1B52D84C7F7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7267575" y="171451"/>
+          <a:ext cx="2553067" cy="2442064"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>495694</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>134795</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C0E2428-8399-0F37-4E1B-DCAD50A7047F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4505325" y="190501"/>
+          <a:ext cx="2724544" cy="2420794"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -586,10 +744,10 @@
         <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -597,7 +755,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="3">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="C4" s="3">
         <v>0</v>
@@ -611,13 +769,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="2">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C5" s="2">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="D5" s="2">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -625,13 +783,13 @@
         <v>6</v>
       </c>
       <c r="B6" s="3">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C6" s="3">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="D6" s="3">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -639,13 +797,13 @@
         <v>7</v>
       </c>
       <c r="B7" s="2">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C7" s="2">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="D7" s="2">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -653,13 +811,13 @@
         <v>8</v>
       </c>
       <c r="B8" s="3">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C8" s="3">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="D8" s="3">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -667,13 +825,13 @@
         <v>9</v>
       </c>
       <c r="B9" s="2">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C9" s="2">
+        <v>31</v>
+      </c>
+      <c r="D9" s="2">
         <v>15</v>
-      </c>
-      <c r="D9" s="2">
-        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -681,13 +839,13 @@
         <v>10</v>
       </c>
       <c r="B10" s="3">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C10" s="3">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="D10" s="3">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -703,13 +861,13 @@
         <v>2</v>
       </c>
       <c r="B12" s="3">
-        <v>212</v>
+        <v>242</v>
       </c>
       <c r="C12" s="3">
-        <v>56</v>
+        <v>124</v>
       </c>
       <c r="D12" s="3">
-        <v>32</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -720,10 +878,10 @@
         <v>76</v>
       </c>
       <c r="C13" s="2">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="D13" s="2">
-        <v>16</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -738,12 +896,12 @@
     </row>
     <row r="17" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
@@ -767,5 +925,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>